<commit_message>
update notebooks and scenario mapping and tableau dashboards
</commit_message>
<xml_diff>
--- a/ssp_modeling/scenario_mapping/ssp_bulgaria_transformation_jan_19.xlsx
+++ b/ssp_modeling/scenario_mapping/ssp_bulgaria_transformation_jan_19.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tony/Documents/sisepuede_modeling/ssp_bulgaria/ssp_modeling/scenario_mapping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FFCFA8A-8D92-F84C-8596-8730688A0B07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC6427A6-459C-704D-A025-DBD450D76589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="260" yWindow="620" windowWidth="37500" windowHeight="19660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6540" yWindow="22260" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -1635,7 +1635,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1782,6 +1782,15 @@
     </xf>
     <xf numFmtId="3" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2235,12 +2244,8 @@
       <c r="N3" s="13">
         <v>12</v>
       </c>
-      <c r="O3" s="16">
-        <v>1</v>
-      </c>
-      <c r="P3" s="16">
-        <v>1</v>
-      </c>
+      <c r="O3" s="16"/>
+      <c r="P3" s="16"/>
       <c r="Q3" s="10"/>
       <c r="R3" s="11"/>
       <c r="S3" s="11"/>
@@ -2966,95 +2971,91 @@
       <c r="R19" s="11"/>
       <c r="S19" s="11"/>
     </row>
-    <row r="20" spans="1:21" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="12" t="s">
+    <row r="20" spans="1:21" s="53" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="42" t="s">
         <v>51</v>
       </c>
-      <c r="B20" s="26" t="s">
+      <c r="B20" s="42" t="s">
         <v>51</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="42" t="s">
         <v>64</v>
       </c>
-      <c r="D20" s="12" t="s">
+      <c r="D20" s="42" t="s">
         <v>65</v>
       </c>
-      <c r="E20" s="12" t="s">
+      <c r="E20" s="42" t="s">
         <v>267</v>
       </c>
-      <c r="F20" s="12" t="s">
+      <c r="F20" s="42" t="s">
         <v>268</v>
       </c>
-      <c r="G20" s="12" t="s">
+      <c r="G20" s="42" t="s">
         <v>412</v>
       </c>
-      <c r="H20" s="12"/>
-      <c r="I20" s="12">
+      <c r="H20" s="42"/>
+      <c r="I20" s="42">
         <v>0</v>
       </c>
-      <c r="J20" s="12">
-        <v>1</v>
-      </c>
-      <c r="K20" s="12"/>
-      <c r="L20" s="12"/>
-      <c r="M20" s="15">
+      <c r="J20" s="42">
+        <v>1</v>
+      </c>
+      <c r="K20" s="42"/>
+      <c r="L20" s="42"/>
+      <c r="M20" s="48">
         <v>0.1</v>
       </c>
-      <c r="N20" s="13">
+      <c r="N20" s="49">
         <v>7</v>
       </c>
-      <c r="O20" s="16"/>
-      <c r="P20" s="16">
-        <v>0.01</v>
-      </c>
-      <c r="Q20" s="10"/>
-      <c r="R20" s="11"/>
-      <c r="S20" s="11"/>
-    </row>
-    <row r="21" spans="1:21" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="12" t="s">
+      <c r="O20" s="43"/>
+      <c r="P20" s="43"/>
+      <c r="Q20" s="51"/>
+      <c r="R20" s="52"/>
+      <c r="S20" s="52"/>
+    </row>
+    <row r="21" spans="1:21" s="53" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="42" t="s">
         <v>51</v>
       </c>
-      <c r="B21" s="26" t="s">
+      <c r="B21" s="42" t="s">
         <v>51</v>
       </c>
-      <c r="C21" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="D21" s="12" t="s">
+      <c r="C21" s="42" t="s">
+        <v>67</v>
+      </c>
+      <c r="D21" s="42" t="s">
         <v>68</v>
       </c>
-      <c r="E21" s="12" t="s">
+      <c r="E21" s="42" t="s">
         <v>269</v>
       </c>
-      <c r="F21" s="12" t="s">
+      <c r="F21" s="42" t="s">
         <v>270</v>
       </c>
-      <c r="G21" s="12" t="s">
+      <c r="G21" s="42" t="s">
         <v>412</v>
       </c>
-      <c r="H21" s="12"/>
-      <c r="I21" s="12">
+      <c r="H21" s="42"/>
+      <c r="I21" s="42">
         <v>0</v>
       </c>
-      <c r="J21" s="12">
-        <v>1</v>
-      </c>
-      <c r="K21" s="12"/>
-      <c r="L21" s="12"/>
-      <c r="M21" s="15">
+      <c r="J21" s="42">
+        <v>1</v>
+      </c>
+      <c r="K21" s="42"/>
+      <c r="L21" s="42"/>
+      <c r="M21" s="48">
         <v>0.1</v>
       </c>
-      <c r="N21" s="13">
+      <c r="N21" s="49">
         <v>7</v>
       </c>
-      <c r="O21" s="16"/>
-      <c r="P21" s="16">
-        <v>0.01</v>
-      </c>
-      <c r="Q21" s="10"/>
-      <c r="R21" s="11"/>
-      <c r="S21" s="11"/>
+      <c r="O21" s="43"/>
+      <c r="P21" s="43"/>
+      <c r="Q21" s="51"/>
+      <c r="R21" s="52"/>
+      <c r="S21" s="52"/>
     </row>
     <row r="22" spans="1:21" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="12" t="s">

</xml_diff>